<commit_message>
nova versao beta dia 13.01
</commit_message>
<xml_diff>
--- a/controle_financeiro.xlsx
+++ b/controle_financeiro.xlsx
@@ -8,6 +8,7 @@
   <sheets>
     <sheet name="Controle" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Categorias" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Config" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -510,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="5.44140625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -555,6 +556,11 @@
           <t>detalhesCartao</t>
         </is>
       </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>investimentos</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="40.2" customHeight="1" thickBot="1">
       <c r="A2" s="2" t="n">
@@ -620,24 +626,29 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D4" t="n">
         <v>13665.21</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>[{"descricao": "teste 3", "valor": -5}, {"descricao": "Planos de Saude", "valor": -946.72}, {"descricao": "IRRF", "valor": -2535.37}, {"descricao": "INSS", "valor": -951.62}, {"descricao": "Sindicato", "valor": -35}, {"descricao": "Seguro de Vida", "valor": -15.58}]</t>
+          <t>[{"descricao": "teste 3", "valor": -5}, {"descricao": "Planos de Saude", "valor": -946.72}, {"descricao": "IRRF", "valor": -2535.37}, {"descricao": "INSS", "valor": -951.62}, {"descricao": "Sindicato", "valor": -35}]</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>[{"pago": true, "descricao": "Escola Yuri", "categoria": "Educação", "valor": 843.18, "tipo": "Despesa"}, {"pago": true, "descricao": "2/95 Cheque Especial Acordo", "categoria": "Dividas", "valor": 137.53, "tipo": "Despesa"}, {"pago": true, "descricao": "Quinto Andar", "categoria": "Moradia", "valor": 2445.19, "tipo": "Despesa"}, {"pago": true, "descricao": "2/71 Cartão Credito Acordo", "categoria": "Dividas", "valor": 770.56, "tipo": "Despesa"}, {"pago": true, "descricao": "Emprestimo Consignado 15/96", "categoria": "Dividas", "valor": 2747.32, "tipo": "Despesa"}, {"pago": true, "descricao": "3/6 Cartão Carrefour", "categoria": "Dividas", "valor": 45.19, "tipo": "Despesa"}, {"pago": true, "descricao": "Fatura Mensal", "categoria": "Cartão Nubank", "valor": 20, "tipo": "Despesa"}]</t>
+          <t>[{"pago": true, "vencimento": "", "descricao": "Escola Yuri", "categoria": "Educação", "valor": 843.18, "tipo": "Despesa"}, {"pago": true, "vencimento": "", "descricao": "2/95 Cheque Especial Acordo", "categoria": "Dividas", "valor": 137.53, "tipo": "Despesa"}, {"pago": true, "vencimento": "", "descricao": "Fatura Mensal", "categoria": "Cartão Nubank", "valor": 89, "tipo": "Despesa"}]</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>[{"cartaoOrigem": "Cartão Nubank", "descricao": "teste", "categoria": "Alimentação", "valor": 8}, {"cartaoOrigem": "Cartão Nubank", "descricao": "teste", "categoria": "Alimentação", "valor": 12}]</t>
+          <t>[{"cartaoOrigem": "Nubank", "descricao": "Amazon", "categoria": "Alimentação", "valor": 89}]</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>[{"nome": "Teste", "tipo": "CDB", "valor": 600}]</t>
         </is>
       </c>
     </row>
@@ -665,7 +676,17 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>[{"pago": false, "descricao": "Emprestimo Consignado 16/96", "categoria": "Dividas", "valor": 2747.32, "tipo": "Despesa"}, {"pago": false, "descricao": "Cheque Especial Acordo 3/95", "categoria": "Dividas", "valor": 137.53, "tipo": "Despesa"}, {"pago": false, "descricao": "Cartão Credito Acordo 3/71", "categoria": "Dividas", "valor": 770.56, "tipo": "Despesa"}, {"pago": false, "descricao": "Cartão Carrefour 4/6", "categoria": "Dividas", "valor": 45.19, "tipo": "Despesa"}, {"pago": false, "descricao": "Aluguel", "categoria": "Moradia", "valor": 2000, "tipo": "Despesa"}, {"pago": false, "descricao": "Escola Yuri", "categoria": "Educação", "valor": 843.18, "tipo": "Despesa"}, {"pago": false, "descricao": "Claro Móvel", "categoria": "Outros", "valor": 54.9, "tipo": "Despesa"}, {"pago": false, "descricao": "Claro Internet", "categoria": "Outros", "valor": 99, "tipo": "Despesa"}, {"pago": false, "descricao": "Gympass", "categoria": "Saúde", "valor": 59, "tipo": "Despesa"}, {"pago": false, "descricao": "Transporte Publico", "categoria": "Transporte", "valor": 153, "tipo": "Despesa"}, {"pago": false, "descricao": "Mercado", "categoria": "Alimentação", "valor": 600, "tipo": "Despesa"}, {"pago": false, "descricao": "Gasolina", "categoria": "Transporte", "valor": 300, "tipo": "Despesa"}, {"pago": false, "descricao": "Seguro Carro 7/7", "categoria": "Transporte", "valor": 254.9, "tipo": "Despesa"}, {"pago": false, "descricao": "CC Nubank", "categoria": "Outros", "valor": 620, "tipo": "Despesa"}]</t>
+          <t>[{"pago": false, "vencimento": "", "descricao": "Emprestimo Consignado 16/96", "categoria": "Dividas", "valor": 2747.32, "tipo": "Despesa"}, {"pago": false, "vencimento": "", "descricao": "Cheque Especial Acordo 3/95", "categoria": "Dividas", "valor": 137.53, "tipo": "Despesa"}, {"pago": false, "vencimento": "", "descricao": "Cartão Credito Acordo 3/71", "categoria": "Dividas", "valor": 770.56, "tipo": "Despesa"}, {"pago": false, "vencimento": "", "descricao": "Cartão Carrefour 4/6", "categoria": "Dividas", "valor": 45.19, "tipo": "Despesa"}, {"pago": false, "vencimento": "", "descricao": "Aluguel", "categoria": "Moradia", "valor": 2000, "tipo": "Despesa"}, {"pago": false, "vencimento": "", "descricao": "Escola Yuri", "categoria": "Educação", "valor": 843.18, "tipo": "Despesa"}, {"pago": false, "vencimento": "", "descricao": "Claro Móvel", "categoria": "Outros", "valor": 54.9, "tipo": "Despesa"}, {"pago": false, "vencimento": "", "descricao": "Claro Internet", "categoria": "Outros", "valor": 99, "tipo": "Despesa"}, {"pago": false, "vencimento": "", "descricao": "Transporte Publico", "categoria": "Transporte", "valor": 153, "tipo": "Despesa"}, {"pago": false, "vencimento": "", "descricao": "Mercado", "categoria": "Alimentação", "valor": 600, "tipo": "Despesa"}, {"pago": false, "vencimento": "", "descricao": "Gasolina", "categoria": "Transporte", "valor": 300, "tipo": "Despesa"}, {"pago": false, "vencimento": "", "descricao": "Fatura Mensal", "categoria": "Cartão Nubank", "valor": 620, "tipo": "Despesa"}, {"pago": false, "vencimento": "2025-12-10", "descricao": "Seguro Carro 7/7", "categoria": "Transporte", "valor": 254.9, "tipo": "Despesa"}]</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>[{"cartaoOrigem": "Nubank", "descricao": "Mochila Kalunga 3/3", "categoria": "Educação", "valor": 149.96}, {"cartaoOrigem": "Nubank", "descricao": "Limite Convertido", "categoria": "Dividas", "valor": 103.99}, {"cartaoOrigem": "Nubank", "descricao": "Ifood", "categoria": "Alimentação", "valor": 57.01}, {"cartaoOrigem": "Nubank", "descricao": "Pizzaria Sahara", "categoria": "Alimentação", "valor": 46}, {"cartaoOrigem": "Nubank", "descricao": "Wellhub", "categoria": "Saúde", "valor": 59.9}, {"cartaoOrigem": "Nubank", "descricao": "Gasolina Portal SBC", "categoria": "Transporte", "valor": 100}, {"cartaoOrigem": "Nubank", "descricao": "Pedagio", "categoria": "Transporte", "valor": 17.8}, {"cartaoOrigem": "Nubank", "descricao": "Mercado Barbosa", "categoria": "Alimentação", "valor": 85.34}]</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>[]</t>
         </is>
       </c>
     </row>
@@ -749,4 +770,32 @@
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.787401575" bottom="0.787401575" header="0.31496062" footer="0.31496062"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Cartoes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>["Nubank", "Santander"]</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
refactor: Migração completa para PostgreSQL + Svelte - Nova arquitetura com autenticação JWT
- Backend: Flask + SQLAlchemy + PostgreSQL
- Frontend: Svelte + Vite com componentes modernos
- Autenticação: Sistema JWT implementado
- Banco de dados: Schema normalizado com 7 tabelas
- Script de migração: Importação de dados do Excel
- Documentação: README e SETUP completos
</commit_message>
<xml_diff>
--- a/controle_financeiro.xlsx
+++ b/controle_financeiro.xlsx
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="5.44140625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -626,7 +626,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
         <v>13665.21</v>
@@ -638,7 +638,7 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>[{"pago": true, "vencimento": "", "descricao": "Escola Yuri", "categoria": "Educação", "valor": 843.18, "tipo": "Despesa"}, {"pago": true, "vencimento": "", "descricao": "2/95 Cheque Especial Acordo", "categoria": "Dividas", "valor": 137.53, "tipo": "Despesa"}, {"pago": true, "vencimento": "", "descricao": "Fatura Mensal", "categoria": "Cartão Nubank", "valor": 89, "tipo": "Despesa"}]</t>
+          <t>[{"pago": true, "vencimento": "", "descricao": "Escola Yuri", "categoria": "Educação", "valor": 843.18, "tipo": "Despesa"}, {"pago": true, "vencimento": "", "descricao": "2/95 Cheque Especial Acordo", "categoria": "Dividas", "valor": 137.53, "tipo": "Despesa"}, {"pago": true, "vencimento": "", "descricao": "Quinto Andar", "categoria": "Moradia", "valor": 2445.19, "tipo": "Despesa"}, {"pago": true, "vencimento": "", "descricao": "2/71 Cartão Credito Acordo", "categoria": "Dividas", "valor": 770.56, "tipo": "Despesa"}, {"pago": true, "vencimento": "", "descricao": "Fatura Mensal", "categoria": "Cartão Nubank", "valor": 89, "tipo": "Despesa"}, {"pago": true, "vencimento": "2025-12-31", "descricao": "Emprestimo Consignado 15/96", "categoria": "Dividas", "valor": 2747.32, "tipo": "Despesa"}]</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -676,7 +676,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>[{"pago": false, "vencimento": "", "descricao": "Emprestimo Consignado 16/96", "categoria": "Dividas", "valor": 2747.32, "tipo": "Despesa"}, {"pago": false, "vencimento": "", "descricao": "Cheque Especial Acordo 3/95", "categoria": "Dividas", "valor": 137.53, "tipo": "Despesa"}, {"pago": false, "vencimento": "", "descricao": "Cartão Credito Acordo 3/71", "categoria": "Dividas", "valor": 770.56, "tipo": "Despesa"}, {"pago": false, "vencimento": "", "descricao": "Cartão Carrefour 4/6", "categoria": "Dividas", "valor": 45.19, "tipo": "Despesa"}, {"pago": false, "vencimento": "", "descricao": "Aluguel", "categoria": "Moradia", "valor": 2000, "tipo": "Despesa"}, {"pago": false, "vencimento": "", "descricao": "Escola Yuri", "categoria": "Educação", "valor": 843.18, "tipo": "Despesa"}, {"pago": false, "vencimento": "", "descricao": "Claro Móvel", "categoria": "Outros", "valor": 54.9, "tipo": "Despesa"}, {"pago": false, "vencimento": "", "descricao": "Claro Internet", "categoria": "Outros", "valor": 99, "tipo": "Despesa"}, {"pago": false, "vencimento": "", "descricao": "Transporte Publico", "categoria": "Transporte", "valor": 153, "tipo": "Despesa"}, {"pago": false, "vencimento": "", "descricao": "Mercado", "categoria": "Alimentação", "valor": 600, "tipo": "Despesa"}, {"pago": false, "vencimento": "", "descricao": "Gasolina", "categoria": "Transporte", "valor": 300, "tipo": "Despesa"}, {"pago": false, "vencimento": "", "descricao": "Fatura Mensal", "categoria": "Cartão Nubank", "valor": 620, "tipo": "Despesa"}, {"pago": false, "vencimento": "2025-12-10", "descricao": "Seguro Carro 7/7", "categoria": "Transporte", "valor": 254.9, "tipo": "Despesa"}]</t>
+          <t>[{"pago": false, "vencimento": "", "descricao": "Cartão Carrefour 4/6", "categoria": "Dividas", "valor": 45.19, "tipo": "Despesa"}, {"pago": false, "vencimento": "", "descricao": "Aluguel", "categoria": "Moradia", "valor": 2000, "tipo": "Despesa"}, {"pago": false, "vencimento": "", "descricao": "Claro Móvel", "categoria": "Outros", "valor": 54.9, "tipo": "Despesa"}, {"pago": false, "vencimento": "", "descricao": "Claro Internet", "categoria": "Outros", "valor": 99, "tipo": "Despesa"}, {"pago": false, "vencimento": "", "descricao": "Transporte Publico", "categoria": "Transporte", "valor": 153, "tipo": "Despesa"}, {"pago": false, "vencimento": "", "descricao": "Mercado", "categoria": "Alimentação", "valor": 600, "tipo": "Despesa"}, {"pago": false, "vencimento": "", "descricao": "Gasolina", "categoria": "Transporte", "valor": 300, "tipo": "Despesa"}, {"pago": false, "vencimento": "", "descricao": "Fatura Mensal", "categoria": "Cartão Nubank", "valor": 620, "tipo": "Despesa"}, {"pago": false, "vencimento": "2025-12-10", "descricao": "Seguro Carro 7/7", "categoria": "Transporte", "valor": 254.9, "tipo": "Despesa"}, {"pago": false, "vencimento": "2026-01-31", "descricao": "Emprestimo Consignado 16/96", "categoria": "Dividas", "valor": 2747.32, "tipo": "Despesa"}, {"pago": false, "vencimento": "2026-02-07", "descricao": "Escola Yuri", "categoria": "Educação", "valor": 843.18, "tipo": "Despesa"}, {"pago": false, "vencimento": "2026-02-05", "descricao": "Cartão Credito Acordo 3/71", "categoria": "Dividas", "valor": 770.56, "tipo": "Despesa"}, {"pago": false, "vencimento": "2026-02-05", "descricao": "Cheque Especial Acordo 3/95", "categoria": "Dividas", "valor": 137.53, "tipo": "Despesa"}, {"pago": false, "vencimento": "2026-01-31", "descricao": "Enel Atrasos", "categoria": "Moradia", "valor": 38.78, "tipo": "Despesa"}, {"pago": false, "vencimento": "2026-02-02", "descricao": "Enel", "categoria": "Moradia", "valor": 196.67, "tipo": "Despesa"}, {"pago": false, "vencimento": "2026-02-02", "descricao": "Material Escola 1/2", "categoria": "Moradia", "valor": 365, "tipo": "Despesa"}]</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -685,6 +685,44 @@
         </is>
       </c>
       <c r="H5" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Março</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>14276.86</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>[{"descricao": "Auxilio Creche Reembolso", "valor": 43.18}, {"descricao": "INSS", "valor": -988.07}, {"descricao": "IRRF", "valor": -2681.68}, {"descricao": "Plano De Saude", "valor": -1340.49}, {"descricao": "Seguro de Vida", "valor": -16.23}, {"descricao": "Empréstimo Consignado", "valor": -2747.32}, {"descricao": "Sindicato", "valor": -35}, {"descricao": "PLR", "valor": 40558.49}, {"descricao": "IRRF sobre PLR", "valor": -7986.78}, {"descricao": "Reembolso Dicidio", "valor": 569.13}, {"descricao": "IIRF Dicidio", "valor": -156.51}, {"descricao": "Sindicato Dicidio", "valor": -35}]</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>[]</t>
         </is>

</xml_diff>